<commit_message>
Update 25MMS5501-NIIT-CISCO-US-Attendance Roster_Splunk Basics_2-4 Mar'26.xlsx
</commit_message>
<xml_diff>
--- a/25MMS5501-NIIT-CISCO-US-Attendance Roster_Splunk Basics_2-4 Mar'26.xlsx
+++ b/25MMS5501-NIIT-CISCO-US-Attendance Roster_Splunk Basics_2-4 Mar'26.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\CISCO_US_02_03_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D08BD82F-0BB7-4B70-9A26-DAB582D821B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0585C1-DC84-4FF7-BA3D-A286F78805F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="51">
   <si>
     <t>Start Date</t>
   </si>
@@ -182,6 +182,12 @@
   </si>
   <si>
     <t>https://cloud.cdp.rpsconsulting.in/console/#/</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -273,7 +279,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -458,15 +464,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -501,7 +498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -533,50 +530,40 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="15" fontId="2" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -587,21 +574,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -895,11 +889,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="30"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -982,147 +976,171 @@
       <c r="B11" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="35">
         <v>46083</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="13">
         <v>46084</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="13">
         <v>46085</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
+      <c r="C12" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="32"/>
+      <c r="E12" s="15"/>
     </row>
     <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
+      <c r="C13" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="32"/>
+      <c r="E13" s="15"/>
     </row>
     <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="26" t="s">
+      <c r="A14" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
+      <c r="C14" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="32"/>
+      <c r="E14" s="15"/>
     </row>
     <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
+      <c r="C15" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="32"/>
+      <c r="E15" s="15"/>
     </row>
     <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
+      <c r="C16" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="32"/>
+      <c r="E16" s="15"/>
     </row>
     <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
+      <c r="C17" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="32"/>
+      <c r="E17" s="15"/>
     </row>
     <row r="18" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
+      <c r="C18" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="32"/>
+      <c r="E18" s="15"/>
     </row>
     <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
+      <c r="C19" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="32"/>
+      <c r="E19" s="15"/>
     </row>
     <row r="20" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="26" t="s">
+      <c r="A20" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
+      <c r="C20" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="32"/>
+      <c r="E20" s="15"/>
     </row>
     <row r="21" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="19"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="20"/>
+      <c r="C21" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" s="33"/>
+      <c r="E21" s="15"/>
     </row>
     <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="26" t="s">
+      <c r="A22" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="27" t="s">
+      <c r="B22" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
+      <c r="C22" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="32"/>
+      <c r="E22" s="15"/>
     </row>
     <row r="23" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="25" t="s">
+      <c r="B23" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="16"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
+      <c r="C23" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="34"/>
+      <c r="E23" s="14"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A12:B23">
@@ -1163,189 +1181,189 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B6" s="35"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="31"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="19"/>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36" t="s">
+      <c r="C9" s="22"/>
+      <c r="D9" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36" t="s">
+      <c r="C10" s="22"/>
+      <c r="D10" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36" t="s">
+      <c r="C11" s="22"/>
+      <c r="D11" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="37" t="s">
+      <c r="E11" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="35" t="s">
+      <c r="B12" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36" t="s">
+      <c r="C12" s="22"/>
+      <c r="D12" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="37" t="s">
+      <c r="E12" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="35" t="s">
+      <c r="B13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="36" t="s">
+      <c r="C13" s="22"/>
+      <c r="D13" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="37" t="s">
+      <c r="E13" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36" t="s">
+      <c r="C14" s="22"/>
+      <c r="D14" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="37" t="s">
+      <c r="E14" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36" t="s">
+      <c r="C15" s="22"/>
+      <c r="D15" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="37" t="s">
+      <c r="E15" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36" t="s">
+      <c r="C16" s="22"/>
+      <c r="D16" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36" t="s">
+      <c r="C17" s="22"/>
+      <c r="D17" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="37" t="s">
+      <c r="E17" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36" t="s">
+      <c r="C18" s="22"/>
+      <c r="D18" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="37" t="s">
+      <c r="E18" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36" t="s">
+      <c r="C19" s="22"/>
+      <c r="D19" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="35" t="s">
+      <c r="B20" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36" t="s">
+      <c r="C20" s="22"/>
+      <c r="D20" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="37" t="s">
+      <c r="E20" s="24" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="33" t="s">
+      <c r="E21" s="21" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>